<commit_message>
KHEO v1.0.1 - Initial solar engineering model
</commit_message>
<xml_diff>
--- a/output/KHEO.xlsx
+++ b/output/KHEO.xlsx
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>15410</v>
+        <v>16685</v>
       </c>
     </row>
     <row r="5">
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>10620</v>
+        <v>11118</v>
       </c>
     </row>
     <row r="6">
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-4790</v>
+        <v>-5567</v>
       </c>
     </row>
     <row r="7">
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.6891628812459442</v>
+        <v>0.6663470182798921</v>
       </c>
     </row>
     <row r="10">
@@ -946,13 +946,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>664</v>
+        <v>1585</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1450</v>
+        <v>1379</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>786</v>
+        <v>-206</v>
       </c>
     </row>
     <row r="5">
@@ -962,13 +962,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>583</v>
+        <v>1418</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1220</v>
+        <v>1245</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>637</v>
+        <v>-173</v>
       </c>
     </row>
     <row r="6">
@@ -978,13 +978,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>632</v>
+        <v>1335</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>930</v>
+        <v>1090</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>298</v>
+        <v>-245</v>
       </c>
     </row>
     <row r="7">
@@ -994,13 +994,13 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>1005</v>
+        <v>1251</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>650</v>
+        <v>867</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-355</v>
+        <v>-384</v>
       </c>
     </row>
     <row r="8">
@@ -1010,13 +1010,13 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>1564</v>
+        <v>1335</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>420</v>
+        <v>589</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-1144</v>
+        <v>-746</v>
       </c>
     </row>
     <row r="9">
@@ -1026,13 +1026,13 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>2413</v>
+        <v>1502</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>310</v>
+        <v>434</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-2103</v>
+        <v>-1068</v>
       </c>
     </row>
     <row r="10">
@@ -1042,13 +1042,13 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>2358</v>
+        <v>1669</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>360</v>
+        <v>500</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-1998</v>
+        <v>-1169</v>
       </c>
     </row>
     <row r="11">
@@ -1058,13 +1058,13 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>2488</v>
+        <v>1585</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>560</v>
+        <v>700</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-1928</v>
+        <v>-885</v>
       </c>
     </row>
     <row r="12">
@@ -1074,13 +1074,13 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1026</v>
+        <v>1335</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>820</v>
+        <v>934</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-206</v>
+        <v>-401</v>
       </c>
     </row>
     <row r="13">
@@ -1090,13 +1090,13 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>1333</v>
+        <v>1251</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1100</v>
+        <v>1123</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-233</v>
+        <v>-128</v>
       </c>
     </row>
     <row r="14">
@@ -1106,13 +1106,13 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>709</v>
+        <v>1168</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>1320</v>
+        <v>1167</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>611</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="15">
@@ -1122,13 +1122,13 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>635</v>
+        <v>1251</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1480</v>
+        <v>1090</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>845</v>
+        <v>-161</v>
       </c>
     </row>
     <row r="16">
@@ -1138,13 +1138,13 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>15410</v>
+        <v>16685</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>10620</v>
+        <v>11118</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-4790</v>
+        <v>-5567</v>
       </c>
     </row>
   </sheetData>
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>15410</v>
+        <v>16685</v>
       </c>
     </row>
     <row r="6">
@@ -1550,7 +1550,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>10620</v>
+        <v>11118</v>
       </c>
     </row>
     <row r="7">
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>0.6891628812459442</v>
+        <v>0.6663470182798921</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
KHEO v1.0.2 - Read monthly usage from CSV
</commit_message>
<xml_diff>
--- a/output/KHEO.xlsx
+++ b/output/KHEO.xlsx
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>16685</v>
+        <v>15410</v>
       </c>
     </row>
     <row r="5">
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-5567</v>
+        <v>-4292</v>
       </c>
     </row>
     <row r="7">
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.6663470182798921</v>
+        <v>0.7214795587280987</v>
       </c>
     </row>
     <row r="10">
@@ -942,193 +942,193 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1585</v>
+        <v>1005</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1379</v>
+        <v>867</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-206</v>
+        <v>-138</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>May</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1418</v>
+        <v>1564</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1245</v>
+        <v>589</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-173</v>
+        <v>-975</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1335</v>
+        <v>2413</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1090</v>
+        <v>434</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-245</v>
+        <v>-1979</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Jul</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>1251</v>
+        <v>2358</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>867</v>
+        <v>500</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-384</v>
+        <v>-1858</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>1335</v>
+        <v>2488</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>589</v>
+        <v>700</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-746</v>
+        <v>-1788</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>1502</v>
+        <v>1026</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>434</v>
+        <v>934</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-1068</v>
+        <v>-92</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Jul</t>
+          <t>Oct</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>1669</v>
+        <v>1333</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>500</v>
+        <v>1123</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-1169</v>
+        <v>-210</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Aug</t>
+          <t>Nov</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>1585</v>
+        <v>709</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>700</v>
+        <v>1167</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-885</v>
+        <v>458</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Dec</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1335</v>
+        <v>635</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>934</v>
+        <v>1090</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-401</v>
+        <v>455</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Oct</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>1251</v>
+        <v>664</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1123</v>
+        <v>1379</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-128</v>
+        <v>715</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Nov</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>1168</v>
+        <v>583</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>1167</v>
+        <v>1245</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-1</v>
+        <v>662</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Dec</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>1251</v>
+        <v>632</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>1090</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-161</v>
+        <v>458</v>
       </c>
     </row>
     <row r="16">
@@ -1138,13 +1138,13 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>16685</v>
+        <v>15410</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>11118</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-5567</v>
+        <v>-4292</v>
       </c>
     </row>
   </sheetData>
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>16685</v>
+        <v>15410</v>
       </c>
     </row>
     <row r="6">
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>0.6663470182798921</v>
+        <v>0.7214795587280987</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Feature 010 - Add roof geometry data file
</commit_message>
<xml_diff>
--- a/output/KHEO.xlsx
+++ b/output/KHEO.xlsx
@@ -456,10 +456,11 @@
   <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="2" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,6 +470,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -518,7 +520,7 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>11118</v>
+        <v>13557</v>
       </c>
     </row>
     <row r="6">
@@ -538,7 +540,7 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-4292</v>
+        <v>-1853</v>
       </c>
     </row>
     <row r="7">
@@ -558,9 +560,11 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.7214795587280987</v>
-      </c>
-    </row>
+        <v>0.8797534068786502</v>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -640,6 +644,8 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
@@ -709,8 +715,8 @@
   <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
@@ -722,6 +728,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -901,13 +908,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -917,6 +927,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -935,6 +946,21 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Direct Use (kWh)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Grid Import (kWh)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Grid Export (kWh)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>Balance (kWh)</t>
         </is>
       </c>
@@ -949,10 +975,19 @@
         <v>1005</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>867</v>
+        <v>1001</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-138</v>
+        <v>350</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>655</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>651</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>-4</v>
       </c>
     </row>
     <row r="5">
@@ -965,10 +1000,19 @@
         <v>1564</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>589</v>
+        <v>742</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-975</v>
+        <v>260</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>1304</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>482</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>-822</v>
       </c>
     </row>
     <row r="6">
@@ -981,10 +1025,19 @@
         <v>2413</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>434</v>
+        <v>539</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-1979</v>
+        <v>189</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>2224</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>-1874</v>
       </c>
     </row>
     <row r="7">
@@ -997,10 +1050,19 @@
         <v>2358</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>500</v>
+        <v>610</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-1858</v>
+        <v>214</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2144</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>396</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>-1748</v>
       </c>
     </row>
     <row r="8">
@@ -1013,10 +1075,19 @@
         <v>2488</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>700</v>
+        <v>822</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-1788</v>
+        <v>288</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>534</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>-1666</v>
       </c>
     </row>
     <row r="9">
@@ -1029,10 +1100,19 @@
         <v>1026</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>934</v>
+        <v>1026</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-92</v>
+        <v>359</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>667</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>667</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1045,10 +1125,19 @@
         <v>1333</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>1123</v>
+        <v>1326</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-210</v>
+        <v>464</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>869</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>862</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>-7</v>
       </c>
     </row>
     <row r="11">
@@ -1061,10 +1150,19 @@
         <v>709</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>1167</v>
+        <v>1488</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>458</v>
+        <v>521</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>188</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>967</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>779</v>
       </c>
     </row>
     <row r="12">
@@ -1077,10 +1175,19 @@
         <v>635</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1090</v>
+        <v>1644</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>455</v>
+        <v>575</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>1069</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>1009</v>
       </c>
     </row>
     <row r="13">
@@ -1093,10 +1200,19 @@
         <v>664</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1379</v>
+        <v>1697</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>715</v>
+        <v>594</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>1103</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>1033</v>
       </c>
     </row>
     <row r="14">
@@ -1109,10 +1225,19 @@
         <v>583</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>1245</v>
+        <v>1389</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>662</v>
+        <v>486</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>903</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>806</v>
       </c>
     </row>
     <row r="15">
@@ -1125,10 +1250,19 @@
         <v>632</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1090</v>
+        <v>1273</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>458</v>
+        <v>446</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>186</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>827</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>641</v>
       </c>
     </row>
     <row r="16">
@@ -1141,11 +1275,18 @@
         <v>15410</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>11118</v>
+        <v>13557</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-4292</v>
-      </c>
+        <v>-1853</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>10664</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>8811</v>
+      </c>
+      <c r="G16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1161,7 +1302,7 @@
   <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -1174,6 +1315,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1181,6 +1323,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -1237,8 +1380,8 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1250,6 +1393,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1307,8 +1451,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1320,6 +1464,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1394,10 +1539,10 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1407,6 +1552,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1513,8 +1659,8 @@
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1526,6 +1672,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1533,6 +1680,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1550,7 +1698,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>11118</v>
+        <v>13557</v>
       </c>
     </row>
     <row r="7">
@@ -1560,9 +1708,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>0.7214795587280987</v>
-      </c>
-    </row>
+        <v>0.8797534068786502</v>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
@@ -1570,6 +1719,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Version 1.2.0 - Add Solar worksheet
</commit_message>
<xml_diff>
--- a/output/KHEO.xlsx
+++ b/output/KHEO.xlsx
@@ -1278,7 +1278,7 @@
         <v>13557</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-1853</v>
+        <v>4746</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>10664</v>
@@ -1286,7 +1286,9 @@
       <c r="F16" s="3" t="n">
         <v>8811</v>
       </c>
-      <c r="G16" s="3" t="n"/>
+      <c r="G16" s="3" t="n">
+        <v>-1853</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1299,13 +1301,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1317,25 +1321,92 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Version 1.0 uses estimated monthly solar generation.</t>
         </is>
       </c>
-    </row>
-    <row r="4"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Panels</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Panel Rating (kW)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Array Size (kW)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Tilt (°)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Azimuth (°)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>45</v>
+      </c>
+    </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>A future version will calculate generation from:</t>
         </is>
       </c>
+      <c r="B5" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>315</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>• Christchurch irradiation</t>
         </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>10.81</v>
       </c>
     </row>
     <row r="7">

</xml_diff>